<commit_message>
Ajuste no script de contratos
</commit_message>
<xml_diff>
--- a/SAP/CONTRATOS/Planilhas/Contratos.xlsx
+++ b/SAP/CONTRATOS/Planilhas/Contratos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junio\OneDrive\Área de Trabalho\Documentos\Scripts Github\automations\SAP\CONTRATOS\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\SAP\CONTRATOS\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A829D494-46C6-4F4E-8A2E-ACFA8D5EFEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFF1E09-CEE5-4F07-B33F-8066B1CFD0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C88C6739-E8C1-4ABA-A295-F3266F31B792}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{C88C6739-E8C1-4ABA-A295-F3266F31B792}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>ID_CONTRATO</t>
   </si>
@@ -81,53 +81,35 @@
     <t>MK</t>
   </si>
   <si>
-    <t>31.12.2024</t>
-  </si>
-  <si>
     <t>CIF</t>
   </si>
   <si>
-    <t>São Paulo</t>
-  </si>
-  <si>
-    <t>50.00</t>
-  </si>
-  <si>
-    <t>I1</t>
-  </si>
-  <si>
     <t>BRL</t>
   </si>
   <si>
-    <t>15.50</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>WK</t>
-  </si>
-  <si>
-    <t>30.06.2025</t>
-  </si>
-  <si>
-    <t>FOB</t>
-  </si>
-  <si>
-    <t>Rio de Janeiro</t>
-  </si>
-  <si>
-    <t>120.00</t>
-  </si>
-  <si>
-    <t>I0</t>
+    <t>MI01</t>
+  </si>
+  <si>
+    <t>I14</t>
+  </si>
+  <si>
+    <t>31.10.2026</t>
+  </si>
+  <si>
+    <t>P080</t>
+  </si>
+  <si>
+    <t>MATRIZ</t>
+  </si>
+  <si>
+    <t>C8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,17 +118,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -181,19 +171,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -210,9 +201,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -250,7 +241,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -356,7 +347,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -498,7 +489,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -507,26 +498,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6B4A2AF-DF9C-4A3E-801E-187E389FE683}">
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,161 +572,160 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>100500</v>
+        <v>1030687</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="3">
+        <v>20000991</v>
+      </c>
+      <c r="L2" s="2">
         <v>1000</v>
       </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1100</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="1">
-        <v>99001</v>
-      </c>
-      <c r="L2" s="2">
-        <v>100</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>21</v>
+      <c r="M2" s="2">
+        <v>2.52</v>
       </c>
       <c r="N2" s="2">
         <v>1</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>100500</v>
+        <v>1030687</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3">
+        <v>20001626</v>
+      </c>
+      <c r="L3" s="2">
         <v>1000</v>
       </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1100</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="1">
-        <v>99002</v>
-      </c>
-      <c r="L3" s="2">
-        <v>300</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>24</v>
+      <c r="M3" s="2">
+        <v>1.1100000000000001</v>
       </c>
       <c r="N3" s="2">
         <v>1</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="2"/>
+      <c r="P3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="Q3" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2">
-        <v>200300</v>
+        <v>1030687</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="2">
-        <v>2000</v>
-      </c>
-      <c r="E4" s="2">
-        <v>2</v>
+        <v>17</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3">
+        <v>20001627</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="M4" s="2">
         <v>2</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" s="1">
-        <v>88005</v>
-      </c>
-      <c r="L4" s="2">
-        <v>50</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="N4" s="2">
         <v>1</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId1" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{4B98B7FC-1CC0-4D3C-B6BF-3C6E87028F70}"/>
+    <hyperlink ref="K3" r:id="rId2" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{2A0D511D-07A5-45D3-B358-F3A5049F9C37}"/>
+    <hyperlink ref="K4" r:id="rId3" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{8BD7C034-9356-45C8-B16D-B99C4C4C76DD}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajuste de script de contratos
</commit_message>
<xml_diff>
--- a/SAP/CONTRATOS/Planilhas/Contratos.xlsx
+++ b/SAP/CONTRATOS/Planilhas/Contratos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junio\OneDrive\Área de Trabalho\Documentos\Scripts Github\automations\SAP\CONTRATOS\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A829D494-46C6-4F4E-8A2E-ACFA8D5EFEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0FE43D-046F-4BCF-81A4-2F991CE2F150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C88C6739-E8C1-4ABA-A295-F3266F31B792}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="24">
   <si>
     <t>ID_CONTRATO</t>
   </si>
@@ -72,62 +72,38 @@
     <t>Classificação Contabil</t>
   </si>
   <si>
-    <t>Cód. Imposto</t>
-  </si>
-  <si>
     <t>Moeda</t>
   </si>
   <si>
     <t>MK</t>
   </si>
   <si>
-    <t>31.12.2024</t>
-  </si>
-  <si>
     <t>CIF</t>
   </si>
   <si>
-    <t>São Paulo</t>
-  </si>
-  <si>
-    <t>50.00</t>
-  </si>
-  <si>
-    <t>I1</t>
-  </si>
-  <si>
     <t>BRL</t>
   </si>
   <si>
-    <t>15.50</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>WK</t>
-  </si>
-  <si>
-    <t>30.06.2025</t>
-  </si>
-  <si>
-    <t>FOB</t>
-  </si>
-  <si>
-    <t>Rio de Janeiro</t>
-  </si>
-  <si>
-    <t>120.00</t>
-  </si>
-  <si>
-    <t>I0</t>
+    <t>MI01</t>
+  </si>
+  <si>
+    <t>I14</t>
+  </si>
+  <si>
+    <t>31.10.2026</t>
+  </si>
+  <si>
+    <t>P080</t>
+  </si>
+  <si>
+    <t>MATRIZ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,17 +112,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -181,19 +165,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -506,27 +491,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6B4A2AF-DF9C-4A3E-801E-187E389FE683}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,165 +561,152 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>100500</v>
+        <v>1030687</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2">
+      <c r="J2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="3">
+        <v>20000991</v>
+      </c>
+      <c r="L2" s="2">
         <v>1000</v>
       </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1100</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="1">
-        <v>99001</v>
-      </c>
-      <c r="L2" s="2">
-        <v>100</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>21</v>
+      <c r="M2" s="2">
+        <v>2.52</v>
       </c>
       <c r="N2" s="2">
         <v>1</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>100500</v>
+        <v>1030687</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2">
+      <c r="J3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="3">
+        <v>20001626</v>
+      </c>
+      <c r="L3" s="2">
         <v>1000</v>
       </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1100</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="1">
-        <v>99002</v>
-      </c>
-      <c r="L3" s="2">
-        <v>300</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>24</v>
+      <c r="M3" s="2">
+        <v>1.1100000000000001</v>
       </c>
       <c r="N3" s="2">
         <v>1</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2">
-        <v>200300</v>
+        <v>1030687</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="2">
-        <v>2000</v>
-      </c>
-      <c r="E4" s="2">
-        <v>2</v>
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="3">
+        <v>20001627</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="M4" s="2">
         <v>2</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" s="1">
-        <v>88005</v>
-      </c>
-      <c r="L4" s="2">
-        <v>50</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="N4" s="2">
         <v>1</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId1" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{4B98B7FC-1CC0-4D3C-B6BF-3C6E87028F70}"/>
+    <hyperlink ref="K3" r:id="rId2" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{2A0D511D-07A5-45D3-B358-F3A5049F9C37}"/>
+    <hyperlink ref="K4" r:id="rId3" display="https://s4qas.sap.avivar.com.br/sap/bc/ui2/flp?sap-client=300&amp;sap-language=PT" xr:uid="{8BD7C034-9356-45C8-B16D-B99C4C4C76DD}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>